<commit_message>
i will create and make changes in that code
</commit_message>
<xml_diff>
--- a/ExcelFiles/Combined_data_BSE.xlsx
+++ b/ExcelFiles/Combined_data_BSE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Equity Data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Corporate Governance" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Board_Members" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Peer_Annual Data" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equity Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Governance" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Board_Members" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peer_Annual Data" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z17"/>
+  <dimension ref="A1:Z18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2002,25 +2002,17 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>1040.95</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>1040.95</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>1065.00</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>1012.00</t>
-        </is>
+      <c r="A17" t="n">
+        <v>1040.95</v>
+      </c>
+      <c r="B17" t="n">
+        <v>1040.95</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1065</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1012</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -2037,15 +2029,11 @@
           <t>779.75</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>4099</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>42.58</t>
-        </is>
+      <c r="H17" t="n">
+        <v>4099</v>
+      </c>
+      <c r="I17" t="n">
+        <v>42.58</v>
       </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
@@ -2058,25 +2046,17 @@
           <t>472.16</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>33.95</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>84.53</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>10.63</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>5.00</t>
-        </is>
+      <c r="M17" t="n">
+        <v>33.95</v>
+      </c>
+      <c r="N17" t="n">
+        <v>84.53</v>
+      </c>
+      <c r="O17" t="n">
+        <v>10.63</v>
+      </c>
+      <c r="P17" t="n">
+        <v>5</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2098,15 +2078,11 @@
           <t>Auto Components &amp; Equipments</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>30.66</t>
-        </is>
-      </c>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>3.26</t>
-        </is>
+      <c r="U17" t="n">
+        <v>30.66</v>
+      </c>
+      <c r="V17" t="n">
+        <v>3.26</v>
       </c>
       <c r="W17" t="inlineStr">
         <is>
@@ -2118,12 +2094,134 @@
           <t>Auto Components &amp; Equipments</t>
         </is>
       </c>
-      <c r="Y17" t="inlineStr">
-        <is>
-          <t>1860</t>
-        </is>
+      <c r="Y17" t="n">
+        <v>1860</v>
       </c>
       <c r="Z17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>233.70</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>238.05</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>242.45</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>228.80</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>230.84</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>404.40</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>212.30</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>4322</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>9.97</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>605.72</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>260.46</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>16.51</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>16.36</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>15.03</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>10.00</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Listed</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>B /T+1</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>Meat Products including Poultry</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>13.93</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>2.09</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>6874</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2136,7 +2234,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X257"/>
+  <dimension ref="A1:X268"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27352,856 +27450,2002 @@
       </c>
     </row>
     <row r="251">
-      <c r="A251" t="inlineStr">
+      <c r="A251" t="n">
+        <v>1</v>
+      </c>
+      <c r="B251" t="n">
+        <v>50950</v>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Executive Director,MD</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I251" t="inlineStr"/>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K251" t="inlineStr">
+        <is>
+          <t>01-11-2014</t>
+        </is>
+      </c>
+      <c r="L251" t="inlineStr">
+        <is>
+          <t>01-11-2022</t>
+        </is>
+      </c>
+      <c r="M251" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N251" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O251" t="n">
+        <v>2</v>
+      </c>
+      <c r="P251" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q251" t="n">
+        <v>2</v>
+      </c>
+      <c r="R251" t="n">
+        <v>0</v>
+      </c>
+      <c r="S251" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T251" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U251" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V251" t="inlineStr">
+        <is>
+          <t>Mr Shailendrajit Rai</t>
+        </is>
+      </c>
+      <c r="W251" t="inlineStr">
+        <is>
+          <t>Alicon-castalloy-limited</t>
+        </is>
+      </c>
+      <c r="X251" t="inlineStr">
+        <is>
+          <t>Auto Components &amp; Equipments</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="n">
+        <v>2</v>
+      </c>
+      <c r="B252" t="n">
+        <v>2628162</v>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Non-Executive - Non Independent Director</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t>18-02-2023</t>
+        </is>
+      </c>
+      <c r="K252" t="inlineStr">
+        <is>
+          <t>29-10-2002</t>
+        </is>
+      </c>
+      <c r="L252" t="inlineStr">
+        <is>
+          <t>29-10-2002</t>
+        </is>
+      </c>
+      <c r="M252" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N252" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O252" t="n">
+        <v>2</v>
+      </c>
+      <c r="P252" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q252" t="n">
+        <v>0</v>
+      </c>
+      <c r="R252" t="n">
+        <v>0</v>
+      </c>
+      <c r="S252" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T252" t="inlineStr">
+        <is>
+          <t>The Company has passed a resolution via postal ballot dt January 17, 2023 for continuation of Directorship of Mr. Junichi Suzuki (DIN : 02628162) as Non-Executive Director.</t>
+        </is>
+      </c>
+      <c r="U252" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V252" t="inlineStr">
+        <is>
+          <t>Mr Junichi Suzuki</t>
+        </is>
+      </c>
+      <c r="W252" t="inlineStr">
+        <is>
+          <t>Alicon-castalloy-limited</t>
+        </is>
+      </c>
+      <c r="X252" t="inlineStr">
+        <is>
+          <t>Auto Components &amp; Equipments</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="n">
+        <v>3</v>
+      </c>
+      <c r="B253" t="n">
+        <v>50999</v>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Non-Executive - Non Independent Director</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I253" t="inlineStr"/>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K253" t="inlineStr">
+        <is>
+          <t>29-09-2014</t>
+        </is>
+      </c>
+      <c r="L253" t="inlineStr">
+        <is>
+          <t>29-09-2014</t>
+        </is>
+      </c>
+      <c r="M253" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N253" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O253" t="n">
+        <v>1</v>
+      </c>
+      <c r="P253" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q253" t="n">
+        <v>0</v>
+      </c>
+      <c r="R253" t="n">
+        <v>0</v>
+      </c>
+      <c r="S253" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T253" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U253" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V253" t="inlineStr">
+        <is>
+          <t>Mrs Pamela Rai</t>
+        </is>
+      </c>
+      <c r="W253" t="inlineStr">
+        <is>
+          <t>Alicon-castalloy-limited</t>
+        </is>
+      </c>
+      <c r="X253" t="inlineStr">
+        <is>
+          <t>Auto Components &amp; Equipments</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="n">
+        <v>4</v>
+      </c>
+      <c r="B254" t="n">
+        <v>2370729</v>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Non-Executive - Independent Director,Chairperson</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I254" t="inlineStr"/>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K254" t="inlineStr">
+        <is>
+          <t>30-04-2015</t>
+        </is>
+      </c>
+      <c r="L254" t="inlineStr">
+        <is>
+          <t>30-04-2020</t>
+        </is>
+      </c>
+      <c r="M254" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N254" t="inlineStr">
+        <is>
+          <t>107.00</t>
+        </is>
+      </c>
+      <c r="O254" t="n">
+        <v>2</v>
+      </c>
+      <c r="P254" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q254" t="n">
+        <v>2</v>
+      </c>
+      <c r="R254" t="n">
+        <v>0</v>
+      </c>
+      <c r="S254" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T254" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U254" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V254" t="inlineStr">
+        <is>
+          <t>Mr Ajay Nanavati</t>
+        </is>
+      </c>
+      <c r="W254" t="inlineStr">
+        <is>
+          <t>Alicon-castalloy-limited</t>
+        </is>
+      </c>
+      <c r="X254" t="inlineStr">
+        <is>
+          <t>Auto Components &amp; Equipments</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="n">
+        <v>5</v>
+      </c>
+      <c r="B255" t="n">
+        <v>4168</v>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Non-Executive - Independent Director</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I255" t="inlineStr"/>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K255" t="inlineStr">
+        <is>
+          <t>15-10-2019</t>
+        </is>
+      </c>
+      <c r="L255" t="inlineStr">
+        <is>
+          <t>15-10-2019</t>
+        </is>
+      </c>
+      <c r="M255" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N255" t="inlineStr">
+        <is>
+          <t>53.00</t>
+        </is>
+      </c>
+      <c r="O255" t="n">
+        <v>3</v>
+      </c>
+      <c r="P255" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q255" t="n">
+        <v>0</v>
+      </c>
+      <c r="R255" t="n">
+        <v>3</v>
+      </c>
+      <c r="S255" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T255" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U255" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V255" t="inlineStr">
+        <is>
+          <t>Mrs Veena Mankar</t>
+        </is>
+      </c>
+      <c r="W255" t="inlineStr">
+        <is>
+          <t>Alicon-castalloy-limited</t>
+        </is>
+      </c>
+      <c r="X255" t="inlineStr">
+        <is>
+          <t>Auto Components &amp; Equipments</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="n">
+        <v>6</v>
+      </c>
+      <c r="B256" t="n">
+        <v>1259252</v>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Non-Executive - Non Independent Director</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I256" t="inlineStr"/>
+      <c r="J256" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K256" t="inlineStr">
+        <is>
+          <t>26-03-2024</t>
+        </is>
+      </c>
+      <c r="L256" t="inlineStr">
+        <is>
+          <t>26-03-2024</t>
+        </is>
+      </c>
+      <c r="M256" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N256" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O256" t="n">
+        <v>1</v>
+      </c>
+      <c r="P256" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q256" t="n">
+        <v>0</v>
+      </c>
+      <c r="R256" t="n">
+        <v>0</v>
+      </c>
+      <c r="S256" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T256" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U256" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V256" t="inlineStr">
+        <is>
+          <t>Mr Jitendra H Panjabi</t>
+        </is>
+      </c>
+      <c r="W256" t="inlineStr">
+        <is>
+          <t>Alicon-castalloy-limited</t>
+        </is>
+      </c>
+      <c r="X256" t="inlineStr">
+        <is>
+          <t>Auto Components &amp; Equipments</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="n">
+        <v>7</v>
+      </c>
+      <c r="B257" t="n">
+        <v>10617020</v>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Non-Executive - Independent Director</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I257" t="inlineStr"/>
+      <c r="J257" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K257" t="inlineStr">
+        <is>
+          <t>08-08-2024</t>
+        </is>
+      </c>
+      <c r="L257" t="inlineStr">
+        <is>
+          <t>08-08-2024</t>
+        </is>
+      </c>
+      <c r="M257" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N257" t="inlineStr">
+        <is>
+          <t>60.00</t>
+        </is>
+      </c>
+      <c r="O257" t="n">
+        <v>1</v>
+      </c>
+      <c r="P257" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q257" t="n">
+        <v>0</v>
+      </c>
+      <c r="R257" t="n">
+        <v>0</v>
+      </c>
+      <c r="S257" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T257" t="inlineStr">
+        <is>
+          <t>Mr. Alfred Knecht is a Deutsh i.e. a foreigner and therefore does not hold PAN.</t>
+        </is>
+      </c>
+      <c r="U257" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V257" t="inlineStr">
+        <is>
+          <t>Mr Alfred Heinrich Knecht</t>
+        </is>
+      </c>
+      <c r="W257" t="inlineStr">
+        <is>
+          <t>Alicon-castalloy-limited</t>
+        </is>
+      </c>
+      <c r="X257" t="inlineStr">
+        <is>
+          <t>Auto Components &amp; Equipments</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B251" t="inlineStr">
-        <is>
-          <t>00050950</t>
-        </is>
-      </c>
-      <c r="C251" t="inlineStr">
-        <is>
-          <t>Executive Director,MD</t>
-        </is>
-      </c>
-      <c r="D251" t="inlineStr">
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>00002380</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Executive Director,Chairperson related to Promoter</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E251" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F251" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G251" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H251" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="I251" t="inlineStr">
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I258" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="J251" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K251" t="inlineStr">
-        <is>
-          <t>01-11-2014</t>
-        </is>
-      </c>
-      <c r="L251" t="inlineStr">
-        <is>
-          <t>01-11-2022</t>
-        </is>
-      </c>
-      <c r="M251" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N251" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O251" t="inlineStr">
+      <c r="J258" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K258" t="inlineStr">
+        <is>
+          <t>25-06-2006</t>
+        </is>
+      </c>
+      <c r="L258" t="inlineStr">
+        <is>
+          <t>25-06-2021</t>
+        </is>
+      </c>
+      <c r="M258" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N258" t="inlineStr">
+        <is>
+          <t>42.06</t>
+        </is>
+      </c>
+      <c r="O258" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P258" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q258" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R258" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S258" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T258" t="inlineStr"/>
+      <c r="U258" t="inlineStr"/>
+      <c r="V258" t="inlineStr">
+        <is>
+          <t>Mr SKM MAEILANANDHAN</t>
+        </is>
+      </c>
+      <c r="W258" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="X258" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="P251" t="inlineStr">
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>00002384</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Executive Director,CEO-MD</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J259" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K259" t="inlineStr">
+        <is>
+          <t>25-06-2006</t>
+        </is>
+      </c>
+      <c r="L259" t="inlineStr">
+        <is>
+          <t>25-06-2022</t>
+        </is>
+      </c>
+      <c r="M259" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N259" t="inlineStr">
+        <is>
+          <t>30.06</t>
+        </is>
+      </c>
+      <c r="O259" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P259" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="Q251" t="inlineStr">
+      <c r="Q259" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R259" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S259" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T259" t="inlineStr"/>
+      <c r="U259" t="inlineStr"/>
+      <c r="V259" t="inlineStr">
+        <is>
+          <t>Mr SKM SHREE SHIVKUMAR</t>
+        </is>
+      </c>
+      <c r="W259" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="X259" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>00002390</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Non-Executive - Non Independent Director</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J260" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K260" t="inlineStr">
+        <is>
+          <t>29-10-2010</t>
+        </is>
+      </c>
+      <c r="L260" t="inlineStr">
+        <is>
+          <t>29-10-2010</t>
+        </is>
+      </c>
+      <c r="M260" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N260" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O260" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P260" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q260" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R260" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S260" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T260" t="inlineStr"/>
+      <c r="U260" t="inlineStr"/>
+      <c r="V260" t="inlineStr">
+        <is>
+          <t>Mrs S KUMUTAAVALLI</t>
+        </is>
+      </c>
+      <c r="W260" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="X260" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>09469919</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Executive Director</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K261" t="inlineStr">
+        <is>
+          <t>02-08-2023</t>
+        </is>
+      </c>
+      <c r="L261" t="inlineStr">
+        <is>
+          <t>04-12-2023</t>
+        </is>
+      </c>
+      <c r="M261" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N261" t="inlineStr">
+        <is>
+          <t>12.19</t>
+        </is>
+      </c>
+      <c r="O261" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P261" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q261" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R261" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S261" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T261" t="inlineStr"/>
+      <c r="U261" t="inlineStr"/>
+      <c r="V261" t="inlineStr">
+        <is>
+          <t>Mr SK SHARATH RAM</t>
+        </is>
+      </c>
+      <c r="W261" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="X261" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>05170759</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Non-Executive - Independent Director,Shareholder Director</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J262" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K262" t="inlineStr">
+        <is>
+          <t>27-01-2015</t>
+        </is>
+      </c>
+      <c r="L262" t="inlineStr">
+        <is>
+          <t>27-01-2020</t>
+        </is>
+      </c>
+      <c r="M262" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N262" t="inlineStr">
+        <is>
+          <t>59.04</t>
+        </is>
+      </c>
+      <c r="O262" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P262" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q262" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R262" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S262" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T262" t="inlineStr"/>
+      <c r="U262" t="inlineStr"/>
+      <c r="V262" t="inlineStr">
+        <is>
+          <t>Mr D VENKATESWARAN</t>
+        </is>
+      </c>
+      <c r="W262" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="X262" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>00124793</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>Non-Executive - Independent Director,Shareholder Director</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J263" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K263" t="inlineStr">
+        <is>
+          <t>31-07-2019</t>
+        </is>
+      </c>
+      <c r="L263" t="inlineStr">
+        <is>
+          <t>31-07-2024</t>
+        </is>
+      </c>
+      <c r="M263" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N263" t="inlineStr">
+        <is>
+          <t>5.00</t>
+        </is>
+      </c>
+      <c r="O263" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P263" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q263" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R263" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S263" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T263" t="inlineStr"/>
+      <c r="U263" t="inlineStr"/>
+      <c r="V263" t="inlineStr">
+        <is>
+          <t>Mr TN THIRUKUMAR</t>
+        </is>
+      </c>
+      <c r="W263" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="X263" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>08521023</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>Non-Executive - Independent Director,Shareholder Director</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J264" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K264" t="inlineStr">
+        <is>
+          <t>31-07-2019</t>
+        </is>
+      </c>
+      <c r="L264" t="inlineStr">
+        <is>
+          <t>31-07-2024</t>
+        </is>
+      </c>
+      <c r="M264" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N264" t="inlineStr">
+        <is>
+          <t>5.00</t>
+        </is>
+      </c>
+      <c r="O264" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P264" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q264" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R264" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S264" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T264" t="inlineStr"/>
+      <c r="U264" t="inlineStr"/>
+      <c r="V264" t="inlineStr">
+        <is>
+          <t>Mr GN JAYARAM</t>
+        </is>
+      </c>
+      <c r="W264" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="X264" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>00505804</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>Non-Executive - Independent Director,Shareholder Director</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J265" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K265" t="inlineStr">
+        <is>
+          <t>07-08-2024</t>
+        </is>
+      </c>
+      <c r="L265" t="inlineStr">
+        <is>
+          <t>07-08-2024</t>
+        </is>
+      </c>
+      <c r="M265" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N265" t="inlineStr">
+        <is>
+          <t>4.24</t>
+        </is>
+      </c>
+      <c r="O265" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P265" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q265" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R265" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S265" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T265" t="inlineStr"/>
+      <c r="U265" t="inlineStr"/>
+      <c r="V265" t="inlineStr">
+        <is>
+          <t>Mr RR SATHIYAMURTHI</t>
+        </is>
+      </c>
+      <c r="W265" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="X265" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>00077439</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Non-Executive - Independent Director,Shareholder Director</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J266" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K266" t="inlineStr">
+        <is>
+          <t>07-08-2024</t>
+        </is>
+      </c>
+      <c r="L266" t="inlineStr">
+        <is>
+          <t>07-08-2024</t>
+        </is>
+      </c>
+      <c r="M266" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N266" t="inlineStr">
+        <is>
+          <t>4.24</t>
+        </is>
+      </c>
+      <c r="O266" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P266" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q266" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R266" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S266" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T266" t="inlineStr"/>
+      <c r="U266" t="inlineStr"/>
+      <c r="V266" t="inlineStr">
+        <is>
+          <t>Mr AHAMED SHEIK MOHIDEEN KHADER MOHIDEEN</t>
+        </is>
+      </c>
+      <c r="W266" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="X266" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>00150883</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Non-Executive - Independent Director,Shareholder Director</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K267" t="inlineStr">
+        <is>
+          <t>07-08-2024</t>
+        </is>
+      </c>
+      <c r="L267" t="inlineStr">
+        <is>
+          <t>07-08-2024</t>
+        </is>
+      </c>
+      <c r="M267" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N267" t="inlineStr">
+        <is>
+          <t>4.24</t>
+        </is>
+      </c>
+      <c r="O267" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P267" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q267" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R267" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S267" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T267" t="inlineStr"/>
+      <c r="U267" t="inlineStr"/>
+      <c r="V267" t="inlineStr">
+        <is>
+          <t>Mr VIKRAM RAMAKRISHNAN</t>
+        </is>
+      </c>
+      <c r="W267" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="X267" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>05354239</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Non-Executive - Nominee Director</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K268" t="inlineStr">
+        <is>
+          <t>07-08-2024</t>
+        </is>
+      </c>
+      <c r="L268" t="inlineStr">
+        <is>
+          <t>07-08-2024</t>
+        </is>
+      </c>
+      <c r="M268" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N268" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O268" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="R251" t="inlineStr">
+      <c r="P268" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="S251" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T251" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="U251" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V251" t="inlineStr">
-        <is>
-          <t>Mr Shailendrajit Rai</t>
-        </is>
-      </c>
-      <c r="W251" t="inlineStr">
-        <is>
-          <t>Alicon-castalloy-limited</t>
-        </is>
-      </c>
-      <c r="X251" t="inlineStr">
-        <is>
-          <t>Auto Components &amp; Equipments</t>
-        </is>
-      </c>
-    </row>
-    <row r="252">
-      <c r="A252" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B252" t="inlineStr">
-        <is>
-          <t>02628162</t>
-        </is>
-      </c>
-      <c r="C252" t="inlineStr">
-        <is>
-          <t>Non-Executive - Non Independent Director</t>
-        </is>
-      </c>
-      <c r="D252" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E252" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F252" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G252" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H252" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="I252" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J252" t="inlineStr">
-        <is>
-          <t>18-02-2023</t>
-        </is>
-      </c>
-      <c r="K252" t="inlineStr">
-        <is>
-          <t>29-10-2002</t>
-        </is>
-      </c>
-      <c r="L252" t="inlineStr">
-        <is>
-          <t>29-10-2002</t>
-        </is>
-      </c>
-      <c r="M252" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N252" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O252" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="P252" t="inlineStr">
+      <c r="Q268" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="Q252" t="inlineStr">
+      <c r="R268" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="R252" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="S252" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T252" t="inlineStr">
-        <is>
-          <t>The Company has passed a resolution via postal ballot dt January 17, 2023 for continuation of Directorship of Mr. Junichi Suzuki (DIN : 02628162) as Non-Executive Director.</t>
-        </is>
-      </c>
-      <c r="U252" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V252" t="inlineStr">
-        <is>
-          <t>Mr Junichi Suzuki</t>
-        </is>
-      </c>
-      <c r="W252" t="inlineStr">
-        <is>
-          <t>Alicon-castalloy-limited</t>
-        </is>
-      </c>
-      <c r="X252" t="inlineStr">
-        <is>
-          <t>Auto Components &amp; Equipments</t>
-        </is>
-      </c>
-    </row>
-    <row r="253">
-      <c r="A253" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B253" t="inlineStr">
-        <is>
-          <t>00050999</t>
-        </is>
-      </c>
-      <c r="C253" t="inlineStr">
-        <is>
-          <t>Non-Executive - Non Independent Director</t>
-        </is>
-      </c>
-      <c r="D253" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E253" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F253" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G253" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H253" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="I253" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="J253" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K253" t="inlineStr">
-        <is>
-          <t>29-09-2014</t>
-        </is>
-      </c>
-      <c r="L253" t="inlineStr">
-        <is>
-          <t>29-09-2014</t>
-        </is>
-      </c>
-      <c r="M253" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N253" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O253" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="P253" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="Q253" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="R253" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="S253" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T253" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="U253" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V253" t="inlineStr">
-        <is>
-          <t>Mrs Pamela Rai</t>
-        </is>
-      </c>
-      <c r="W253" t="inlineStr">
-        <is>
-          <t>Alicon-castalloy-limited</t>
-        </is>
-      </c>
-      <c r="X253" t="inlineStr">
-        <is>
-          <t>Auto Components &amp; Equipments</t>
-        </is>
-      </c>
-    </row>
-    <row r="254">
-      <c r="A254" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B254" t="inlineStr">
-        <is>
-          <t>02370729</t>
-        </is>
-      </c>
-      <c r="C254" t="inlineStr">
-        <is>
-          <t>Non-Executive - Independent Director,Chairperson</t>
-        </is>
-      </c>
-      <c r="D254" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E254" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F254" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G254" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H254" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="I254" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="J254" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K254" t="inlineStr">
-        <is>
-          <t>30-04-2015</t>
-        </is>
-      </c>
-      <c r="L254" t="inlineStr">
-        <is>
-          <t>30-04-2020</t>
-        </is>
-      </c>
-      <c r="M254" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N254" t="inlineStr">
-        <is>
-          <t>107.00</t>
-        </is>
-      </c>
-      <c r="O254" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="P254" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="Q254" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="R254" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="S254" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T254" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="U254" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V254" t="inlineStr">
-        <is>
-          <t>Mr Ajay Nanavati</t>
-        </is>
-      </c>
-      <c r="W254" t="inlineStr">
-        <is>
-          <t>Alicon-castalloy-limited</t>
-        </is>
-      </c>
-      <c r="X254" t="inlineStr">
-        <is>
-          <t>Auto Components &amp; Equipments</t>
-        </is>
-      </c>
-    </row>
-    <row r="255">
-      <c r="A255" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B255" t="inlineStr">
-        <is>
-          <t>00004168</t>
-        </is>
-      </c>
-      <c r="C255" t="inlineStr">
-        <is>
-          <t>Non-Executive - Independent Director</t>
-        </is>
-      </c>
-      <c r="D255" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E255" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F255" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G255" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H255" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="I255" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="J255" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K255" t="inlineStr">
-        <is>
-          <t>15-10-2019</t>
-        </is>
-      </c>
-      <c r="L255" t="inlineStr">
-        <is>
-          <t>15-10-2019</t>
-        </is>
-      </c>
-      <c r="M255" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N255" t="inlineStr">
-        <is>
-          <t>53.00</t>
-        </is>
-      </c>
-      <c r="O255" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="P255" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="Q255" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="R255" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="S255" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T255" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="U255" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V255" t="inlineStr">
-        <is>
-          <t>Mrs Veena Mankar</t>
-        </is>
-      </c>
-      <c r="W255" t="inlineStr">
-        <is>
-          <t>Alicon-castalloy-limited</t>
-        </is>
-      </c>
-      <c r="X255" t="inlineStr">
-        <is>
-          <t>Auto Components &amp; Equipments</t>
-        </is>
-      </c>
-    </row>
-    <row r="256">
-      <c r="A256" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B256" t="inlineStr">
-        <is>
-          <t>01259252</t>
-        </is>
-      </c>
-      <c r="C256" t="inlineStr">
-        <is>
-          <t>Non-Executive - Non Independent Director</t>
-        </is>
-      </c>
-      <c r="D256" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E256" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F256" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G256" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H256" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="I256" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="J256" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K256" t="inlineStr">
-        <is>
-          <t>26-03-2024</t>
-        </is>
-      </c>
-      <c r="L256" t="inlineStr">
-        <is>
-          <t>26-03-2024</t>
-        </is>
-      </c>
-      <c r="M256" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N256" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O256" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="P256" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="Q256" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="R256" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="S256" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T256" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="U256" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V256" t="inlineStr">
-        <is>
-          <t>Mr Jitendra H Panjabi</t>
-        </is>
-      </c>
-      <c r="W256" t="inlineStr">
-        <is>
-          <t>Alicon-castalloy-limited</t>
-        </is>
-      </c>
-      <c r="X256" t="inlineStr">
-        <is>
-          <t>Auto Components &amp; Equipments</t>
-        </is>
-      </c>
-    </row>
-    <row r="257">
-      <c r="A257" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B257" t="inlineStr">
-        <is>
-          <t>10617020</t>
-        </is>
-      </c>
-      <c r="C257" t="inlineStr">
-        <is>
-          <t>Non-Executive - Independent Director</t>
-        </is>
-      </c>
-      <c r="D257" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E257" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F257" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G257" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H257" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="I257" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="J257" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K257" t="inlineStr">
-        <is>
-          <t>08-08-2024</t>
-        </is>
-      </c>
-      <c r="L257" t="inlineStr">
-        <is>
-          <t>08-08-2024</t>
-        </is>
-      </c>
-      <c r="M257" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N257" t="inlineStr">
-        <is>
-          <t>60.00</t>
-        </is>
-      </c>
-      <c r="O257" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="P257" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="Q257" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="R257" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="S257" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T257" t="inlineStr">
-        <is>
-          <t>Mr. Alfred Knecht is a Deutsh i.e. a foreigner and therefore does not hold PAN.</t>
-        </is>
-      </c>
-      <c r="U257" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V257" t="inlineStr">
-        <is>
-          <t>Mr Alfred Heinrich Knecht</t>
-        </is>
-      </c>
-      <c r="W257" t="inlineStr">
-        <is>
-          <t>Alicon-castalloy-limited</t>
-        </is>
-      </c>
-      <c r="X257" t="inlineStr">
-        <is>
-          <t>Auto Components &amp; Equipments</t>
+      <c r="S268" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T268" t="inlineStr"/>
+      <c r="U268" t="inlineStr"/>
+      <c r="V268" t="inlineStr">
+        <is>
+          <t>Mr K VIVEKANANDAN</t>
+        </is>
+      </c>
+      <c r="W268" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="X268" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
         </is>
       </c>
     </row>
@@ -28216,7 +29460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H257"/>
+  <dimension ref="A1:H268"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38222,296 +39466,744 @@
       </c>
     </row>
     <row r="251">
-      <c r="A251" t="inlineStr">
+      <c r="A251" t="n">
+        <v>1</v>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Mr Shailendrajit Rai</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Executive Director,MD</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>01-11-2014</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>01-11-2022</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>Alicon-castalloy-limited</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>Auto Components &amp; Equipments</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="n">
+        <v>2</v>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Mr Junichi Suzuki</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Non-Executive - Non Independent Director</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>29-10-2002</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>29-10-2002</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>Alicon-castalloy-limited</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>Auto Components &amp; Equipments</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="n">
+        <v>3</v>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Mrs Pamela Rai</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Non-Executive - Non Independent Director</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>29-09-2014</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>29-09-2014</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>Alicon-castalloy-limited</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>Auto Components &amp; Equipments</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="n">
+        <v>4</v>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Mr Ajay Nanavati</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Non-Executive - Independent Director,Chairperson</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>30-04-2015</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>30-04-2020</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>Alicon-castalloy-limited</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>Auto Components &amp; Equipments</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="n">
+        <v>5</v>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Mrs Veena Mankar</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Non-Executive - Independent Director</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>15-10-2019</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>15-10-2019</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>Alicon-castalloy-limited</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>Auto Components &amp; Equipments</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="n">
+        <v>6</v>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Mr Jitendra H Panjabi</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Non-Executive - Non Independent Director</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>26-03-2024</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>26-03-2024</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>Alicon-castalloy-limited</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>Auto Components &amp; Equipments</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="n">
+        <v>7</v>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Mr Alfred Heinrich Knecht</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Non-Executive - Independent Director</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>08-08-2024</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>08-08-2024</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>Alicon-castalloy-limited</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>Auto Components &amp; Equipments</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B251" t="inlineStr">
-        <is>
-          <t>Mr Shailendrajit Rai</t>
-        </is>
-      </c>
-      <c r="C251" t="inlineStr">
-        <is>
-          <t>Executive Director,MD</t>
-        </is>
-      </c>
-      <c r="D251" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="E251" t="inlineStr">
-        <is>
-          <t>01-11-2014</t>
-        </is>
-      </c>
-      <c r="F251" t="inlineStr">
-        <is>
-          <t>01-11-2022</t>
-        </is>
-      </c>
-      <c r="G251" t="inlineStr">
-        <is>
-          <t>Alicon-castalloy-limited</t>
-        </is>
-      </c>
-      <c r="H251" t="inlineStr">
-        <is>
-          <t>Auto Components &amp; Equipments</t>
-        </is>
-      </c>
-    </row>
-    <row r="252">
-      <c r="A252" t="inlineStr">
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Mr SKM MAEILANANDHAN</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Executive Director,Chairperson related to Promoter</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>25-06-2006</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>25-06-2021</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B252" t="inlineStr">
-        <is>
-          <t>Mr Junichi Suzuki</t>
-        </is>
-      </c>
-      <c r="C252" t="inlineStr">
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Mr SKM SHREE SHIVKUMAR</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Executive Director,CEO-MD</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>25-06-2006</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>25-06-2022</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Mrs S KUMUTAAVALLI</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
         <is>
           <t>Non-Executive - Non Independent Director</t>
         </is>
       </c>
-      <c r="D252" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="E252" t="inlineStr">
-        <is>
-          <t>29-10-2002</t>
-        </is>
-      </c>
-      <c r="F252" t="inlineStr">
-        <is>
-          <t>29-10-2002</t>
-        </is>
-      </c>
-      <c r="G252" t="inlineStr">
-        <is>
-          <t>Alicon-castalloy-limited</t>
-        </is>
-      </c>
-      <c r="H252" t="inlineStr">
-        <is>
-          <t>Auto Components &amp; Equipments</t>
-        </is>
-      </c>
-    </row>
-    <row r="253">
-      <c r="A253" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B253" t="inlineStr">
-        <is>
-          <t>Mrs Pamela Rai</t>
-        </is>
-      </c>
-      <c r="C253" t="inlineStr">
-        <is>
-          <t>Non-Executive - Non Independent Director</t>
-        </is>
-      </c>
-      <c r="D253" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="E253" t="inlineStr">
-        <is>
-          <t>29-09-2014</t>
-        </is>
-      </c>
-      <c r="F253" t="inlineStr">
-        <is>
-          <t>29-09-2014</t>
-        </is>
-      </c>
-      <c r="G253" t="inlineStr">
-        <is>
-          <t>Alicon-castalloy-limited</t>
-        </is>
-      </c>
-      <c r="H253" t="inlineStr">
-        <is>
-          <t>Auto Components &amp; Equipments</t>
-        </is>
-      </c>
-    </row>
-    <row r="254">
-      <c r="A254" t="inlineStr">
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>29-10-2010</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>29-10-2010</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B254" t="inlineStr">
-        <is>
-          <t>Mr Ajay Nanavati</t>
-        </is>
-      </c>
-      <c r="C254" t="inlineStr">
-        <is>
-          <t>Non-Executive - Independent Director,Chairperson</t>
-        </is>
-      </c>
-      <c r="D254" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="E254" t="inlineStr">
-        <is>
-          <t>30-04-2015</t>
-        </is>
-      </c>
-      <c r="F254" t="inlineStr">
-        <is>
-          <t>30-04-2020</t>
-        </is>
-      </c>
-      <c r="G254" t="inlineStr">
-        <is>
-          <t>Alicon-castalloy-limited</t>
-        </is>
-      </c>
-      <c r="H254" t="inlineStr">
-        <is>
-          <t>Auto Components &amp; Equipments</t>
-        </is>
-      </c>
-    </row>
-    <row r="255">
-      <c r="A255" t="inlineStr">
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Mr SK SHARATH RAM</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Executive Director</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>02-08-2023</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>04-12-2023</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B255" t="inlineStr">
-        <is>
-          <t>Mrs Veena Mankar</t>
-        </is>
-      </c>
-      <c r="C255" t="inlineStr">
-        <is>
-          <t>Non-Executive - Independent Director</t>
-        </is>
-      </c>
-      <c r="D255" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="E255" t="inlineStr">
-        <is>
-          <t>15-10-2019</t>
-        </is>
-      </c>
-      <c r="F255" t="inlineStr">
-        <is>
-          <t>15-10-2019</t>
-        </is>
-      </c>
-      <c r="G255" t="inlineStr">
-        <is>
-          <t>Alicon-castalloy-limited</t>
-        </is>
-      </c>
-      <c r="H255" t="inlineStr">
-        <is>
-          <t>Auto Components &amp; Equipments</t>
-        </is>
-      </c>
-    </row>
-    <row r="256">
-      <c r="A256" t="inlineStr">
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Mr D VENKATESWARAN</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Non-Executive - Independent Director,Shareholder Director</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>27-01-2015</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>27-01-2020</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B256" t="inlineStr">
-        <is>
-          <t>Mr Jitendra H Panjabi</t>
-        </is>
-      </c>
-      <c r="C256" t="inlineStr">
-        <is>
-          <t>Non-Executive - Non Independent Director</t>
-        </is>
-      </c>
-      <c r="D256" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="E256" t="inlineStr">
-        <is>
-          <t>26-03-2024</t>
-        </is>
-      </c>
-      <c r="F256" t="inlineStr">
-        <is>
-          <t>26-03-2024</t>
-        </is>
-      </c>
-      <c r="G256" t="inlineStr">
-        <is>
-          <t>Alicon-castalloy-limited</t>
-        </is>
-      </c>
-      <c r="H256" t="inlineStr">
-        <is>
-          <t>Auto Components &amp; Equipments</t>
-        </is>
-      </c>
-    </row>
-    <row r="257">
-      <c r="A257" t="inlineStr">
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Mr TN THIRUKUMAR</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>Non-Executive - Independent Director,Shareholder Director</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>31-07-2019</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>31-07-2024</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B257" t="inlineStr">
-        <is>
-          <t>Mr Alfred Heinrich Knecht</t>
-        </is>
-      </c>
-      <c r="C257" t="inlineStr">
-        <is>
-          <t>Non-Executive - Independent Director</t>
-        </is>
-      </c>
-      <c r="D257" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="E257" t="inlineStr">
-        <is>
-          <t>08-08-2024</t>
-        </is>
-      </c>
-      <c r="F257" t="inlineStr">
-        <is>
-          <t>08-08-2024</t>
-        </is>
-      </c>
-      <c r="G257" t="inlineStr">
-        <is>
-          <t>Alicon-castalloy-limited</t>
-        </is>
-      </c>
-      <c r="H257" t="inlineStr">
-        <is>
-          <t>Auto Components &amp; Equipments</t>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Mr GN JAYARAM</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>Non-Executive - Independent Director,Shareholder Director</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>31-07-2019</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>31-07-2024</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Mr RR SATHIYAMURTHI</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>Non-Executive - Independent Director,Shareholder Director</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>07-08-2024</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>07-08-2024</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Mr AHAMED SHEIK MOHIDEEN KHADER MOHIDEEN</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Non-Executive - Independent Director,Shareholder Director</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>07-08-2024</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>07-08-2024</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Mr VIKRAM RAMAKRISHNAN</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Non-Executive - Independent Director,Shareholder Director</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>07-08-2024</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>07-08-2024</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Mr K VIVEKANANDAN</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Non-Executive - Nominee Director</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>07-08-2024</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>07-08-2024</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
         </is>
       </c>
     </row>
@@ -38526,7 +40218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q101"/>
+  <dimension ref="A1:Q105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -45635,10 +47327,8 @@
           <t>1,036.95</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>-0.38</t>
-        </is>
+      <c r="C98" t="n">
+        <v>-0.38</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
@@ -45655,35 +47345,23 @@
           <t>45.83</t>
         </is>
       </c>
-      <c r="G98" t="inlineStr">
-        <is>
-          <t>8.06</t>
-        </is>
-      </c>
-      <c r="H98" t="inlineStr">
-        <is>
-          <t>5.00</t>
-        </is>
-      </c>
-      <c r="I98" t="inlineStr">
-        <is>
-          <t>12.47</t>
-        </is>
-      </c>
-      <c r="J98" t="inlineStr">
-        <is>
-          <t>3.29</t>
-        </is>
-      </c>
-      <c r="K98" t="inlineStr">
-        <is>
-          <t>28.44</t>
-        </is>
-      </c>
-      <c r="L98" t="inlineStr">
-        <is>
-          <t>74.62</t>
-        </is>
+      <c r="G98" t="n">
+        <v>8.06</v>
+      </c>
+      <c r="H98" t="n">
+        <v>5</v>
+      </c>
+      <c r="I98" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="J98" t="n">
+        <v>3.29</v>
+      </c>
+      <c r="K98" t="n">
+        <v>28.44</v>
+      </c>
+      <c r="L98" t="n">
+        <v>74.62</v>
       </c>
       <c r="M98" t="inlineStr">
         <is>
@@ -45722,10 +47400,8 @@
           <t>34,987.50</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>0.90</t>
-        </is>
+      <c r="C99" t="n">
+        <v>0.9</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -45742,35 +47418,23 @@
           <t>2,490.50</t>
         </is>
       </c>
-      <c r="G99" t="inlineStr">
-        <is>
-          <t>29.50</t>
-        </is>
-      </c>
-      <c r="H99" t="inlineStr">
-        <is>
-          <t>10.00</t>
-        </is>
-      </c>
-      <c r="I99" t="inlineStr">
-        <is>
-          <t>21.89</t>
-        </is>
-      </c>
-      <c r="J99" t="inlineStr">
-        <is>
-          <t>14.89</t>
-        </is>
-      </c>
-      <c r="K99" t="inlineStr">
-        <is>
-          <t>844.40</t>
-        </is>
-      </c>
-      <c r="L99" t="inlineStr">
-        <is>
-          <t>989.83</t>
-        </is>
+      <c r="G99" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="H99" t="n">
+        <v>10</v>
+      </c>
+      <c r="I99" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="J99" t="n">
+        <v>14.89</v>
+      </c>
+      <c r="K99" t="n">
+        <v>844.4</v>
+      </c>
+      <c r="L99" t="n">
+        <v>989.83</v>
       </c>
       <c r="M99" t="inlineStr">
         <is>
@@ -45809,10 +47473,8 @@
           <t>90.72</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>-0.74</t>
-        </is>
+      <c r="C100" t="n">
+        <v>-0.74</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
@@ -45829,35 +47491,23 @@
           <t>30.85</t>
         </is>
       </c>
-      <c r="G100" t="inlineStr">
-        <is>
-          <t>13.53</t>
-        </is>
-      </c>
-      <c r="H100" t="inlineStr">
-        <is>
-          <t>1.00</t>
-        </is>
-      </c>
-      <c r="I100" t="inlineStr">
-        <is>
-          <t>11.48</t>
-        </is>
-      </c>
-      <c r="J100" t="inlineStr">
-        <is>
-          <t>1.87</t>
-        </is>
-      </c>
-      <c r="K100" t="inlineStr">
-        <is>
-          <t>2.28</t>
-        </is>
-      </c>
-      <c r="L100" t="inlineStr">
-        <is>
-          <t>9.96</t>
-        </is>
+      <c r="G100" t="n">
+        <v>13.53</v>
+      </c>
+      <c r="H100" t="n">
+        <v>1</v>
+      </c>
+      <c r="I100" t="n">
+        <v>11.48</v>
+      </c>
+      <c r="J100" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="K100" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="L100" t="n">
+        <v>9.960000000000001</v>
       </c>
       <c r="M100" t="inlineStr">
         <is>
@@ -45896,10 +47546,8 @@
           <t>500.00</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>-1.59</t>
-        </is>
+      <c r="C101" t="n">
+        <v>-1.59</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
@@ -45916,59 +47564,395 @@
           <t>145.46</t>
         </is>
       </c>
-      <c r="G101" t="inlineStr">
-        <is>
-          <t>24.14</t>
-        </is>
-      </c>
-      <c r="H101" t="inlineStr">
+      <c r="G101" t="n">
+        <v>24.14</v>
+      </c>
+      <c r="H101" t="n">
+        <v>10</v>
+      </c>
+      <c r="I101" t="n">
+        <v>20.59</v>
+      </c>
+      <c r="J101" t="n">
+        <v>9.529999999999999</v>
+      </c>
+      <c r="K101" t="n">
+        <v>60.26</v>
+      </c>
+      <c r="L101" t="n">
+        <v>90.28</v>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>725.00</t>
+        </is>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>421.48</t>
+        </is>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>Alicon-castalloy-limited</t>
+        </is>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>Auto Components &amp; Equipments</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>SKMEGGPROD</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>230.05</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>-1.56</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Mar - 24</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>689.95</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>83.91</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>26.33</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
         <is>
           <t>10.00</t>
         </is>
       </c>
-      <c r="I101" t="inlineStr">
-        <is>
-          <t>20.59</t>
-        </is>
-      </c>
-      <c r="J101" t="inlineStr">
-        <is>
-          <t>9.53</t>
-        </is>
-      </c>
-      <c r="K101" t="inlineStr">
-        <is>
-          <t>60.26</t>
-        </is>
-      </c>
-      <c r="L101" t="inlineStr">
-        <is>
-          <t>90.28</t>
-        </is>
-      </c>
-      <c r="M101" t="inlineStr">
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>19.46</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>12.16</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>31.87</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>36.24</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="N101" t="inlineStr">
-        <is>
-          <t>725.00</t>
-        </is>
-      </c>
-      <c r="O101" t="inlineStr">
-        <is>
-          <t>421.48</t>
-        </is>
-      </c>
-      <c r="P101" t="inlineStr">
-        <is>
-          <t>Alicon-castalloy-limited</t>
-        </is>
-      </c>
-      <c r="Q101" t="inlineStr">
-        <is>
-          <t>Auto Components &amp; Equipments</t>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>404.40</t>
+        </is>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>212.30</t>
+        </is>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="Q102" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>HMAAGRO</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>38.85</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>-1.65</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Mar - 24</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>4,665.06</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>110.69</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>50.08</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>3.49</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>2.37</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>2.24</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>2.33</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>83.51</t>
+        </is>
+      </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>38.21</t>
+        </is>
+      </c>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>SIMRAN</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>187.60</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>-3.82</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Mar - 24</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>486.42</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>0.31</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>3.79</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>10.00</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>0.85</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>0.06</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>0.82</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>5.40</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t>269.65</t>
+        </is>
+      </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>105.50</t>
+        </is>
+      </c>
+      <c r="P104" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="Q104" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>OVOBELE</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>107.25</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>0.14</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Mar - 24</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>174.63</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>17.89</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>9.50</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>10.00</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>15.03</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>10.24</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>18.83</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>19.86</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>280.00</t>
+        </is>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>97.60</t>
+        </is>
+      </c>
+      <c r="P105" t="inlineStr">
+        <is>
+          <t>Skm-egg-products-export-(india)-ltd</t>
+        </is>
+      </c>
+      <c r="Q105" t="inlineStr">
+        <is>
+          <t>Meat Products Including Poultry</t>
         </is>
       </c>
     </row>

</xml_diff>